<commit_message>
Compact README, prune dead code, widen degree tokens, flag degree-institution fusions
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/review_workbook_new.xlsx
+++ b/review_workbook_new.xlsx
@@ -12,7 +12,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Scientists'!$A$1:$S$128</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA findings'!$A$1:$E$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA findings'!$A$1:$E$25</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -682,7 +682,7 @@
       <c r="R2" s="5" t="n"/>
       <c r="S2" s="5" t="inlineStr">
         <is>
-          <t>WARN: birth_field_repaired -- birth_date 'November 3, 1893' stripped (no printed trace)</t>
+          <t>WARN: birth_field_repaired -- birth_date 'Jan 3, 1893' stripped (no printed trace)</t>
         </is>
       </c>
     </row>
@@ -733,7 +733,7 @@
       </c>
       <c r="K3" s="8" t="inlineStr">
         <is>
-          <t>January 3, 1846</t>
+          <t>Jan. 3, 1846</t>
         </is>
       </c>
       <c r="L3" s="6" t="n">
@@ -755,7 +755,7 @@
       </c>
       <c r="O3" s="9" t="inlineStr">
         <is>
-          <t>Assoc. Ornith. Union, undated</t>
+          <t>Assoc. ornith, Union, undated</t>
         </is>
       </c>
       <c r="P3" s="9" t="inlineStr">
@@ -815,7 +815,7 @@
       </c>
       <c r="K4" s="12" t="inlineStr">
         <is>
-          <t>August 1, 1879</t>
+          <t>Aug. 1, 1879</t>
         </is>
       </c>
       <c r="L4" s="10" t="n">
@@ -926,10 +926,14 @@
           <t>A.A.
 Psychol. Ass
 S. Soc. Philos. and Psychol.
-Psychological problems of tobacco smoking; intelligence characteristics; personnel studies</t>
-        </is>
-      </c>
-      <c r="Q5" s="5" t="n"/>
+Psychological problems of tobacco smoking</t>
+        </is>
+      </c>
+      <c r="Q5" s="5" t="inlineStr">
+        <is>
+          <t>Intelligence characteristics; personnel studies</t>
+        </is>
+      </c>
       <c r="R5" s="5" t="n"/>
       <c r="S5" s="5" t="inlineStr">
         <is>
@@ -994,6 +998,7 @@
         <is>
           <t>B.A, McMaster, 1907
 M.A, McMaster, 1909
+study, Illinois, 1910-1912
 Ph.D, Illinois, 1912</t>
         </is>
       </c>
@@ -1007,8 +1012,7 @@
       </c>
       <c r="O6" s="13" t="inlineStr">
         <is>
-          <t>Fellow, Illinois, 1910-1912
-Research asst, Bur. Standards, 1913</t>
+          <t>Research asst, Bur. Standards, 1913</t>
         </is>
       </c>
       <c r="P6" s="13" t="inlineStr">
@@ -1071,7 +1075,7 @@
       </c>
       <c r="K7" s="4" t="inlineStr">
         <is>
-          <t>January 4, 1870</t>
+          <t>Jan. 4, 1870</t>
         </is>
       </c>
       <c r="L7" s="2" t="n">
@@ -1158,7 +1162,7 @@
       </c>
       <c r="K8" s="12" t="inlineStr">
         <is>
-          <t>September 18, 1881</t>
+          <t>Sept. 18, 1881</t>
         </is>
       </c>
       <c r="L8" s="10" t="n">
@@ -1254,7 +1258,7 @@
       <c r="N9" s="9" t="inlineStr">
         <is>
           <t>Asst. chemist, N. C. Exp. Sta, 1881-1887
-Director and state chemist, N. C. Exp. Sta, 1887-1897
+Director and state chemist, N. C. State Board Health, 1887-1897
 Pres, South. Chem. Co, 1897-1901
 Tech. worker, South. Cotton Oil Co, 1902-1903
 Dist. supt, South. Cotton Oil Co, 1903-1906
@@ -1265,8 +1269,8 @@
       <c r="P9" s="9" t="inlineStr">
         <is>
           <t>A.A.
-Chem. Soc
-Oil Chem. Soc
+Chem. Soc.
+Oil Chem. Soc.
 Ala. Tech. Ass
 Ala. Anthrop. Soc.</t>
         </is>
@@ -1356,8 +1360,8 @@
       </c>
       <c r="P10" s="13" t="inlineStr">
         <is>
-          <t>Chem. Soc
-Harvey Soc
+          <t>Chem. Soc.
+Harvey Soc.
 Chem. Gesell.</t>
         </is>
       </c>
@@ -1437,13 +1441,14 @@
       <c r="P11" s="9" t="inlineStr">
         <is>
           <t>A.A.
-fel. Geol. Soc
-Ass. Petrol. Geol.</t>
+fel. Geol. Soc.
+Ass. Petrol. Geol.
+Coal and oil deposits</t>
         </is>
       </c>
       <c r="Q11" s="9" t="inlineStr">
         <is>
-          <t>Coal and oil deposits; stratigraphy; petroleum</t>
+          <t>Stratigraphy; petroleum</t>
         </is>
       </c>
       <c r="R11" s="9" t="n"/>
@@ -1469,7 +1474,11 @@
           <t>Soil Experiment Fields, Ill.</t>
         </is>
       </c>
-      <c r="F12" s="12" t="n"/>
+      <c r="F12" s="12" t="inlineStr">
+        <is>
+          <t>Soil Experiment Fields</t>
+        </is>
+      </c>
       <c r="G12" s="12" t="inlineStr">
         <is>
           <t>Ill</t>
@@ -1569,7 +1578,7 @@
       </c>
       <c r="K13" s="8" t="inlineStr">
         <is>
-          <t>January 8, 1872</t>
+          <t>Jan. 8, 1872</t>
         </is>
       </c>
       <c r="L13" s="6" t="n">
@@ -1586,9 +1595,9 @@
         <is>
           <t>Teacher, high sch, Minn, 1894-1895
 Instr. math, Iowa, 1895-1898
-Asst. prof, Minnesota, 1900-1902
-Asst. prof, New Hampshire, 1902-1907
-Prof, New Hampshire, 1907-1920
+Instr. math, Minnesota, 1900-1902
+Asst. prof, Minnesota, 1902-1907
+Prof, Minnesota, 1907-1920
 Prof, New Hampshire, 1924-  [current 1927]</t>
         </is>
       </c>
@@ -1600,7 +1609,7 @@
       </c>
       <c r="P13" s="9" t="inlineStr">
         <is>
-          <t>Math. Soc
+          <t>Math. Soc.
 Circolo Mat. di Palermo</t>
         </is>
       </c>
@@ -1663,7 +1672,7 @@
       </c>
       <c r="K14" s="4" t="inlineStr">
         <is>
-          <t>January 26, 1865</t>
+          <t>Jan. 26, 1865</t>
         </is>
       </c>
       <c r="L14" s="2" t="n">
@@ -1682,7 +1691,7 @@
         <is>
           <t>Civil engineer, 1886-1887
 Computer, U. S. Coast and Geod. Surv, 1887-1892
-Docent math. physics, Chicago, 1895
+Docent math. physics, Chicago, 1895-1896
 Instr. geophysics, Chicago, 1896
 Asst. prof. math. and math. physics, Cincinnati, 1897-1899
 Chief div. terrestrial magnetism and inspector magnetic work, U. S. Coast and Geod. Surv, 1899-1906
@@ -1699,21 +1708,21 @@
 Permanent committee on terrestrial magnetism, Int. Meteor. Conf, 1898
 Sec'y, sect. terrestrial magnetism and elec, Int. Geophys. Union, undated
 Chairman, Geophys. Union, 1922-1924
-Chairman and chairman sect. terrestrial magnetism and elec, Geophys. Union, 1920-1926
+V. chairman and chairman sect. terrestrial magnetism and elec, Geophys. Union, 1920-1926
 Nat. Research Council, 1917-  [current 1927]</t>
         </is>
       </c>
       <c r="P14" s="5" t="inlineStr">
         <is>
           <t>A.A. (v. pres, 09)
-Physical Soc
-Astron. Soc
+Physical Soc.
+Astron. Soc.
 Ass. Geog. (v. pres, 09)
-Philos. Soc
-Am. Acad
-Wash. Acad
+Philos. Soc.
+Am. Acad.
+Wash. Acad.
 Wash. Philos. Soc. (pres, 08)
-hon. mem. Cornwall Polytech. Soc
+hon. mem. Cornwall Polytech. Soc.
 Meteor. Gesell
 Soc. Cient. Ant. Alz
 Portugal Geog. Soc
@@ -1727,7 +1736,7 @@
       </c>
       <c r="Q14" s="5" t="inlineStr">
         <is>
-          <t>Lagrange prize, Royal Belgian Acad, 05; Neumayer gold medal, Berlin Gesell. für Erdkunde, 13</t>
+          <t>Terrestrial Magnetism and Atmospheric Elec, 1896-</t>
         </is>
       </c>
       <c r="R14" s="5" t="n"/>
@@ -1793,7 +1802,7 @@
       </c>
       <c r="N15" s="9" t="inlineStr">
         <is>
-          <t>Asst. chemist, bur. chem, U. S. Dept. Agr, 1912-1920
+          <t>Asst. chemist, U. S. Dept. Agr, 1912-1920
 Assoc. chemist, U. S. Dept. Agr, 1920-  [current 1927]</t>
         </is>
       </c>
@@ -1872,7 +1881,7 @@
           <t>Asst. elec. eng, Stanford, 1898-1899
 Practical work, 1899-1900
 Instr. elec. eng, Stanford, 1900-1902
-Asst. prof, Stanford, 1902-  [current 1927]
+Asst. prof, Stanford, 1902-1907
 Consulting engineer, elec. power transmission, 1907-  [current 1927]
 Chief engineer, Calif. Gas and Elec. Corp, 1904-  [current 1927]</t>
         </is>
@@ -1949,7 +1958,8 @@
       <c r="M17" s="9" t="inlineStr">
         <is>
           <t>M.D, Columbia, 1902
-study, Berlin, 1905-1908
+study, Berlin, 1905
+study, Berlin, 1907-1908
 study, Breslau, 1907</t>
         </is>
       </c>
@@ -2140,7 +2150,7 @@
 Instr, Lowthorpe Hort. Sch, 1916-1918
 Asst, Radcliffe, 1917-1918
 C. R. B. Educ. Foundation fellow, Brussels, 1925-1926
-Am-Scandinavica fellow, Lund and Copenhagen, 1926
+Am-Scandinavian fellow, Lund and Copenhagen, 1926
 Sergt, M.C, 1918-1919</t>
         </is>
       </c>
@@ -2302,8 +2312,7 @@
       <c r="M21" s="9" t="inlineStr">
         <is>
           <t>A.B, Kansas, 1900
-A.M, Kansas, 1901
-study, Chicago, 1902-1904</t>
+A.M, Kansas, 1901</t>
         </is>
       </c>
       <c r="N21" s="9" t="inlineStr">
@@ -2315,13 +2324,14 @@
       </c>
       <c r="O21" s="9" t="inlineStr">
         <is>
-          <t>Asst. Univ. of Kans. paleont. exped, Oregon, 1905
+          <t>Fellow, Chicago, 1902-1904
+Asst, Univ. of Kans. paleont. exped, Oregon, 1905
 Entom. exped, Ariz, 1907
 Director zool. exped, Texas, 1908
 Director zool. exped, Wash, 1909
 Staff, Puget Sound Marine Sta, 1909-1916
-Managing ed, 'Kans. Univ. Science Bul', Kansas University, 1910-1914
-Managing ed, 'Kans. Univ. Science Bul', Kansas University, 1919-  [current 1927]</t>
+Managing ed, 'Kans. Univ. Science Bul', 1910-1914
+Managing ed, 'Kans. Univ. Science Bul', 1919-  [current 1927]</t>
         </is>
       </c>
       <c r="P21" s="9" t="inlineStr">
@@ -2339,87 +2349,83 @@
       <c r="S21" s="9" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="n">
+      <c r="A22" s="10" t="n">
         <v>76</v>
       </c>
-      <c r="B22" s="3" t="inlineStr">
+      <c r="B22" s="11" t="inlineStr">
         <is>
           <t>Bausch, Edward</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr">
+      <c r="C22" s="10" t="inlineStr">
         <is>
           <t>*</t>
         </is>
       </c>
-      <c r="D22" s="4" t="n"/>
-      <c r="E22" s="5" t="inlineStr">
+      <c r="D22" s="12" t="n"/>
+      <c r="E22" s="13" t="inlineStr">
         <is>
           <t>Bausch and Lomb Optical Co, Rochester, N. Y</t>
         </is>
       </c>
-      <c r="F22" s="4" t="inlineStr">
+      <c r="F22" s="12" t="inlineStr">
         <is>
           <t>Rochester</t>
         </is>
       </c>
-      <c r="G22" s="4" t="inlineStr">
+      <c r="G22" s="12" t="inlineStr">
         <is>
           <t>N. Y</t>
         </is>
       </c>
-      <c r="H22" s="4" t="inlineStr">
-        <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="I22" s="5" t="inlineStr">
+      <c r="H22" s="12" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="I22" s="13" t="inlineStr">
         <is>
           <t>Optics</t>
         </is>
       </c>
-      <c r="J22" s="5" t="inlineStr">
+      <c r="J22" s="13" t="inlineStr">
         <is>
           <t>Rochester</t>
         </is>
       </c>
-      <c r="K22" s="4" t="inlineStr">
-        <is>
-          <t>Oct. 26, 1854</t>
-        </is>
-      </c>
-      <c r="L22" s="2" t="n">
+      <c r="K22" s="12" t="inlineStr">
+        <is>
+          <t>Sept. 26, 1854</t>
+        </is>
+      </c>
+      <c r="L22" s="10" t="n">
         <v>1854</v>
       </c>
-      <c r="M22" s="5" t="inlineStr">
+      <c r="M22" s="13" t="inlineStr">
         <is>
           <t>study, Cornell, 1875</t>
         </is>
       </c>
-      <c r="N22" s="5" t="inlineStr">
+      <c r="N22" s="13" t="inlineStr">
         <is>
           <t>Pres, Bausch and Lomb Optical Co, undated  [current 1927]</t>
         </is>
       </c>
-      <c r="O22" s="5" t="inlineStr"/>
-      <c r="P22" s="5" t="inlineStr">
+      <c r="O22" s="13" t="inlineStr"/>
+      <c r="P22" s="13" t="inlineStr">
         <is>
           <t>A.A
 Optical Soc
 Micros. Soc</t>
         </is>
       </c>
-      <c r="Q22" s="5" t="inlineStr">
+      <c r="Q22" s="13" t="inlineStr">
         <is>
           <t>Manipulation of the microscope</t>
         </is>
       </c>
-      <c r="R22" s="5" t="n"/>
-      <c r="S22" s="5" t="inlineStr">
-        <is>
-          <t>WARN: birth_month_ocr_mismatch -- extracted 'Oct. 26, 1854' but the OCR text layer reads 'Sept.26,54' -- verify the month on the page image</t>
-        </is>
-      </c>
+      <c r="R22" s="13" t="n"/>
+      <c r="S22" s="13" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="6" t="n">
@@ -2485,7 +2491,7 @@
         <is>
           <t>Asst, Ohio State, 1920-1923
 Head dept. chem, Ottawa (Kans), 1923-1926
-Head dept. chem, Baylor Col. for Women, 1926-  [current 1927]</t>
+Baylor Col. for Women, Baylor Col. for Women, 1926-  [current 1927]</t>
         </is>
       </c>
       <c r="O23" s="9" t="inlineStr"/>
@@ -2556,25 +2562,20 @@
           <t>study, Illinois, 1888-1890
 A.B, Denison, 1893
 A.M, Denison, 1894
-study, Rochester Theol. Sem, 1894-1896
-study, Rochester Theol. Sem, 1897-1898
 Ph.D, Chicago, 1900</t>
         </is>
       </c>
       <c r="N24" s="5" t="inlineStr">
         <is>
           <t>Instr. gymnasium, Denison, 1891-1894
-Instr. biol, Denison, 1894-1896
-Instr. philos, Iowa, 1900-1901
+Instr. biol, Theol. Sem, 1894-1896
+Instr. philos, Iowa, 1897-1898
+Fellow, Chicago, 1898-1900
 Prof, Vassar, 1901-1907
 Prof, Cincinnati, 1907-1908</t>
         </is>
       </c>
-      <c r="O24" s="5" t="inlineStr">
-        <is>
-          <t>Fellow, Denison, 1893-1894</t>
-        </is>
-      </c>
+      <c r="O24" s="5" t="inlineStr"/>
       <c r="P24" s="5" t="inlineStr">
         <is>
           <t>A.A
@@ -2664,11 +2665,10 @@
       </c>
       <c r="O25" s="9" t="inlineStr">
         <is>
-          <t>Summers, special asst, Michigan, 1920
-Office blister rust control, U. S. Dept. Agr, 1919
-Office blister rust control, U. S. Dept. Agr, 1921-1923
-Field asst, office forest path, 1918-1919
-Asst. pathologist, 1924-1925</t>
+          <t>Summers, special asst, Michigan, 1920-1921
+Office blister rust control, U. S. Dept. Agr, 1919-1921
+Field asst, office forest path, U. S. Dept. Agr, 1918-1919
+Asst. pathologist, U. S. Dept. Agr, 1924-1925</t>
         </is>
       </c>
       <c r="P25" s="9" t="inlineStr"/>
@@ -2757,8 +2757,8 @@
       </c>
       <c r="O26" s="13" t="inlineStr">
         <is>
-          <t>Summers, instr, Harvard, 1897-1902
-Radcliffe, Radcliffe, 1902-  [current 1927]</t>
+          <t>Summer instr, Harvard, 1897
+Summer instr, Harvard, 1902-1921</t>
         </is>
       </c>
       <c r="P26" s="13" t="inlineStr">
@@ -2841,8 +2841,8 @@
       </c>
       <c r="N27" s="9" t="inlineStr">
         <is>
-          <t>Asst. psychol. lab, Training Sch. for Feebleminded, Vineland, N. J., 1917-1918
-Psychologist and director child study, Sleighton Farm, Darling, Pa., 1918-1919
+          <t>Asst. psychol. lab, Training Sch. for Feebleminded, Vineland, N. J, 1917-1918
+Psychologist and director child study, Sleighton Farm, Darling, Pa, 1918-1919
 Psychol. examiner child study, dept. pub. instruction, Rochester, 1919-1921
 Psychologist, Board Educ, Cleveland, 1924-  [current 1927]</t>
         </is>
@@ -2850,7 +2850,7 @@
       <c r="O27" s="9" t="inlineStr">
         <is>
           <t>Fellow, Michigan, 1922-1924
-Field worker, Associated Charities, Minneapolis, Minn., 1919</t>
+Field worker, Associated Charities, Minneapolis, Minn, 1919</t>
         </is>
       </c>
       <c r="P27" s="9" t="inlineStr"/>
@@ -2923,7 +2923,7 @@
         <is>
           <t>A.B, Hopkins, 1883
 Ph.D, Hopkins, 1886
-study, Prof. geol, Colby, 1888-1904</t>
+study, Col. geol, Colby, 1888-1904</t>
         </is>
       </c>
       <c r="N28" s="13" t="inlineStr">
@@ -2936,19 +2936,18 @@
       </c>
       <c r="O28" s="13" t="inlineStr">
         <is>
-          <t>Asst. geologist, U. S. Geol. Surv., 1889-1908
-Geologist, U. S. Geol. Surv., 1909-  [current 1927]
-Assoc. ed., Am. Naturalist, 1886-1902
+          <t>Asst. geologist, U. S. Geol. Surv, 1889-1908
+Geologist, U. S. Geol. Surv, 1909-  [current 1927]
+Assoc. ed, Am. Naturalist, 1886-1902
 Reviewer, Neues Jahrbuch, 1890-1908
-Business ed., Econ. Geol., 1905-  [current 1927]</t>
+Business ed, Econ. Geol, 1905-  [current 1927]
+Councillor, A.A., 1919
+Councillor, Soc. Econ. Geol, undated</t>
         </is>
       </c>
       <c r="P28" s="13" t="inlineStr">
         <is>
-          <t>A.A.
-Geol. Soc. (councillor, 19)
-Soc. Econ. Geol. (councillor)
-Ill. Acad. (pres)
+          <t>Ill. Acad. (pres)
 Wash. Geol. Soc
 Chem. Gesell.</t>
         </is>
@@ -3026,7 +3025,7 @@
           <t>Intern med, Hopkins Hosp, 1915-1916
 Instr. path, Hopkins, 1916
 Assoc. prof. path. and bacter, Hopkins, 1920
-Prof. bacter, Sch. med, Rochester, undated  [current 1927]</t>
+Prof. bacter, sch. med, Rochester, undated  [current 1927]</t>
         </is>
       </c>
       <c r="O29" s="9" t="inlineStr"/>
@@ -3103,6 +3102,7 @@
         <is>
           <t>B.A, Oxford, 1908
 M.B, Oxford, 1911
+B.Ch, Oxford, 1911
 M.A, Oxford, 1913
 M.D, Oxford, 1919
 L.R.C.P, ?, 1911</t>
@@ -3112,24 +3112,22 @@
         <is>
           <t>Demonstrator physiol, St. Thomas Hosp, 1910-1911
 Fellow, Magdalen, Oxford, 1912-1920
-Demonstrator path, Christopher Welch, 1913-1915
-Lecturer clin. physiol, Christopher Welch, 1919-1921
+Demonstrator path, St. Thomas Hosp, 1913-1915
+Christopher Welch lecturer clin. physiol, Oxford, 1919-1921
 Prof. physiol, Pennsylvania, 1921-  [current 1927]</t>
         </is>
       </c>
       <c r="O30" s="13" t="inlineStr">
         <is>
-          <t>Radcliffe traveling fellow, 1912-1914
-Cheselden medal, St. Thomas Hosp, 1911
-Mil. Cross, Gt. Britain, 1915
-Order of British Empire, 1918
-Physiol. Soc, Phila. Col. Physicians, undated
-Fellow, Royal Col. Surg, undated</t>
+          <t>Radcliffe traveling fellow, Oxford, 1912-1914</t>
         </is>
       </c>
       <c r="P30" s="13" t="inlineStr">
         <is>
-          <t>British Physiol. Soc.</t>
+          <t>Physiol. Soc
+Phila. Col. Physicians
+fel. Royal Col. Surg
+British Physiol. Soc.</t>
         </is>
       </c>
       <c r="Q30" s="13" t="inlineStr">
@@ -3203,14 +3201,14 @@
       <c r="N31" s="9" t="inlineStr">
         <is>
           <t>Instr. physics, Pennsylvania, 1911-1917
-Asst. research, King's Col, London, 1916-1917
 Asst. prof, Pennsylvania, 1919-1921
 Prof. exp. physics, Pennsylvania, 1921-  [current 1927]</t>
         </is>
       </c>
       <c r="O31" s="9" t="inlineStr">
         <is>
-          <t>Harrison research fellow (London), Pennsylvania, 1915-1916
+          <t>Harrison research fellow, London, 1915-1916
+Asst. research, King's Col, London, 1916-1917
 Capt, C.Eng, 1917-1919</t>
         </is>
       </c>
@@ -3223,7 +3221,7 @@
       </c>
       <c r="Q31" s="9" t="inlineStr">
         <is>
-          <t>Photo-electric and thermionic emissions; ionization potentials</t>
+          <t>Photoelectric and thermionic emissions; ionization potentials</t>
         </is>
       </c>
       <c r="R31" s="9" t="n"/>
@@ -3292,7 +3290,7 @@
       <c r="N32" s="13" t="inlineStr">
         <is>
           <t>Asst, Iowa Col, 1921-1926
-Mellon Inst, Mellon Institute, 1926-  [current 1927]</t>
+Chem, Mellon Inst, 1926-  [current 1927]</t>
         </is>
       </c>
       <c r="O32" s="13" t="inlineStr"/>
@@ -3370,7 +3368,7 @@
       </c>
       <c r="N33" s="9" t="inlineStr">
         <is>
-          <t>Machinist and draftsman, Yale, 1883-1890
+          <t>Machinist and draftsman, 1883-1890
 Asst. physics, Yale, 1891-1894
 Instr, Yale, 1894-1895
 Asst. prof, Yale, 1895-  [current 1927]</t>
@@ -3608,7 +3606,7 @@
       </c>
       <c r="O36" s="13" t="inlineStr">
         <is>
-          <t>Senior mem. board to determine conditions of navigation, U. S. and Europe, 1910-1914
+          <t>Senior mem, board to determine conditions of navigation, U. S. and Europe, 1910-1914
 Board on flood prevention, 1915</t>
         </is>
       </c>
@@ -3677,21 +3675,24 @@
       <c r="M37" s="9" t="inlineStr">
         <is>
           <t>B.S, Minnesota, 1914
-study, Mich. State Col, 1914-1915
-M.S, Mich. State Col, 1915</t>
+M.S, Mich. State Col, 1915
+Ph.D, Illinois, 1918</t>
         </is>
       </c>
       <c r="N37" s="9" t="inlineStr">
         <is>
-          <t>Fellow, Illinois, 1917-1918
-Ph.D, Illinois, 1918
-Asst. bot, Illinois, 1915-1917
+          <t>Asst. bot, Illinois, 1915-1917
 Instr. plant path, Pa. State, 1918-1919
 Asst. prof, Pa. State, 1919-1923
-Assoc. prof, Pa. State, 1923-  [current 1927]</t>
-        </is>
-      </c>
-      <c r="O37" s="9" t="inlineStr"/>
+Assoc. prof, Pa. State, 1925-  [current 1927]</t>
+        </is>
+      </c>
+      <c r="O37" s="9" t="inlineStr">
+        <is>
+          <t>Fellow, Mich. State Col, 1914-1915
+Fellow, Illinois, 1917-1918</t>
+        </is>
+      </c>
       <c r="P37" s="9" t="inlineStr">
         <is>
           <t>A.A.
@@ -3860,13 +3861,13 @@
       </c>
       <c r="O39" s="9" t="inlineStr">
         <is>
-          <t>Chairman, committee on floricul. courses, Soc. Hort. Sci., 1913-1914</t>
+          <t>Chairman, committee on floricult. courses, Soc. Hort. Sci, 1913-1914</t>
         </is>
       </c>
       <c r="P39" s="9" t="inlineStr">
         <is>
           <t>A.A.
-Bot. Soc.
+Bot. Soc
 Soc. Hort. Sci.</t>
         </is>
       </c>
@@ -3920,7 +3921,7 @@
       </c>
       <c r="J40" s="13" t="inlineStr">
         <is>
-          <t>Alrington, Colo.</t>
+          <t>Arlington, Colo.</t>
         </is>
       </c>
       <c r="K40" s="12" t="inlineStr">
@@ -3950,17 +3951,18 @@
       <c r="O40" s="13" t="inlineStr">
         <is>
           <t>Fellow, Pittsburgh, 1914-1916
-Mem. com. committee on nat. lighting, Illum. Eng. Soc., 1921-1924</t>
+Hon. mem. committee on nat. lighting, Illum. Eng. Soc, undated
+Exec. committee, Horol. Inst, 1921-1924</t>
         </is>
       </c>
       <c r="P40" s="13" t="inlineStr">
         <is>
-          <t>Hon. mem. committee on nat. lighting, Illum. Eng. Soc.
-Physical Soc.
-Astron. Soc.
-Horol. Inst.
-Statist. Ass.
-Wash. Acad.
+          <t>Illum. Eng. Soc
+Physical Soc
+Astron. Soc
+Horol. Inst
+Statist. Ass
+Wash. Acad
 Wash. Philos. Soc.</t>
         </is>
       </c>
@@ -4021,13 +4023,13 @@
       <c r="N41" s="5" t="inlineStr">
         <is>
           <t>Asst. geologist, K. T. and Co, 1913
-Consulting geologist, 1913-1914
+Consulting geologist, K. T. and Co, 1913-1914
 Instr. geol. and mining, Stanford, 1914-1915
 Oil and gas inspector, U. S. Bur. Mines, 1915-1916
 Asst. to chief petrol. technologist, U. S. Bur. Mines, 1916-1918
 Special agent, bur. internal revenue, U. S. Treas. Dept, 1918-1919
-Consulting geologist and engineer, 1919-1924
-V. pres, Marland Oil Co., Calif, 1924-  [current 1927]</t>
+Consulting geologist and engineer, Marland Oil Co, Calif, 1919-1924
+V. pres, Marland Oil Co, Calif, 1924-  [current 1927]</t>
         </is>
       </c>
       <c r="O41" s="5" t="inlineStr"/>
@@ -4102,7 +4104,6 @@
         <is>
           <t>Ph.B, Colgate, 1902
 A.M, Princeton, 1905
-study, Princeton, 1909-1910
 Ph.D, Princeton, 1911</t>
         </is>
       </c>
@@ -4185,7 +4186,7 @@
       <c r="M43" s="9" t="inlineStr">
         <is>
           <t>Pharm.D, Scio, 1907
-Ph.B, Scio, 1908
+Ph.B, Columbia, 1908
 A.M, Columbia, 1910
 Ph.D, Columbia, 1911</t>
         </is>
@@ -4204,17 +4205,16 @@
       <c r="O43" s="9" t="inlineStr">
         <is>
           <t>Committee on chem. of med. products, Nat. Research Council, undated
-Sec'y, div. pharmaceut. chem, Chem. Soc., 1915-1919
-Research committee, Pharmaceut. Ass., 1918-  [current 1927]</t>
+Sec'y, div. pharmaceut. chem, Chem. Soc, 1915-1919
+Research committee, Pharmaceut. Ass, 1918</t>
         </is>
       </c>
       <c r="P43" s="9" t="inlineStr">
         <is>
-          <t>Am. Conf. Pharmaceutics, Research, Crop Protection Inst.
+          <t>Am. Conf. Pharmaceutics, Research, Crop Protection Inst
 A.A.
 Chem. Soc.
-Pharmaceut. Ass.
-hon. mem. Ill. Pharmaceut. Ass.</t>
+Pharmaceut. Ass.</t>
         </is>
       </c>
       <c r="Q43" s="9" t="inlineStr">
@@ -4226,59 +4226,59 @@
       <c r="S43" s="9" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" s="10" t="n">
+      <c r="A44" s="2" t="n">
         <v>78</v>
       </c>
-      <c r="B44" s="11" t="inlineStr">
+      <c r="B44" s="3" t="inlineStr">
         <is>
           <t>Beal, J(ames) H(artley)</t>
         </is>
       </c>
-      <c r="C44" s="10" t="inlineStr"/>
-      <c r="D44" s="12" t="inlineStr">
+      <c r="C44" s="2" t="inlineStr"/>
+      <c r="D44" s="4" t="inlineStr">
         <is>
           <t>Dr.</t>
         </is>
       </c>
-      <c r="E44" s="13" t="inlineStr">
+      <c r="E44" s="5" t="inlineStr">
         <is>
           <t>801 W. Nevada St, Urbana, Ill.</t>
         </is>
       </c>
-      <c r="F44" s="12" t="inlineStr">
+      <c r="F44" s="4" t="inlineStr">
         <is>
           <t>Urbana</t>
         </is>
       </c>
-      <c r="G44" s="12" t="inlineStr">
+      <c r="G44" s="4" t="inlineStr">
         <is>
           <t>Ill</t>
         </is>
       </c>
-      <c r="H44" s="12" t="inlineStr">
-        <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="I44" s="13" t="inlineStr">
+      <c r="H44" s="4" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="I44" s="5" t="inlineStr">
         <is>
           <t>Pharmacy</t>
         </is>
       </c>
-      <c r="J44" s="13" t="inlineStr">
+      <c r="J44" s="5" t="inlineStr">
         <is>
           <t>New Philadelphia, Ohio</t>
         </is>
       </c>
-      <c r="K44" s="12" t="inlineStr">
+      <c r="K44" s="4" t="inlineStr">
         <is>
           <t>September 23, 1861</t>
         </is>
       </c>
-      <c r="L44" s="10" t="n">
+      <c r="L44" s="2" t="n">
         <v>1861</v>
       </c>
-      <c r="M44" s="13" t="inlineStr">
+      <c r="M44" s="5" t="inlineStr">
         <is>
           <t>B.S, Scio Col, 1884
 A.B, Scio Col, 1888
@@ -4289,39 +4289,43 @@
 hon. Ph.M, Phila. Col. Pharmacy, 1913</t>
         </is>
       </c>
-      <c r="N44" s="13" t="inlineStr">
+      <c r="N44" s="5" t="inlineStr">
         <is>
           <t>Prof. chem. and dean, dept. pharmacy, Scio Col, 1887-1907
 Prof. applied pharmacy, Pittsburgh, 1902-1911
-Gen. sec'y and ed., Jour. Am. Pharmaceut. Ass, Am. Pharmaceut. Ass., 1911-1914
+Gen. sec'y and ed., 'Jour. Am. Pharmaceut. Ass', Am. Pharmaceut. Ass, 1911-1914
 Director pharmacy research, Illinois, 1914-1918
-Chairman board trustees, U. S. Pharmacopoeia, 1910-  [current 1927]
+Nat. Drug medalist, Illinois, 1919</t>
+        </is>
+      </c>
+      <c r="O44" s="5" t="inlineStr">
+        <is>
+          <t>Chairman board trustees, U. S. Pharmacopoeia, 1910-  [current 1927]
 Mem, W.I.B, 1918
-Nat. Drug medalist, 1919</t>
-        </is>
-      </c>
-      <c r="O44" s="13" t="inlineStr">
-        <is>
-          <t>Pres, Pharmaceut. Ass., 1904
-Pres, Ohio Pharmaceut. Ass., 1898</t>
-        </is>
-      </c>
-      <c r="P44" s="13" t="inlineStr">
+Pres, Pharmaceut. Ass, 1904
+Pres, Ohio Pharmaceut. Ass, 1898</t>
+        </is>
+      </c>
+      <c r="P44" s="5" t="inlineStr">
         <is>
           <t>A.A.
 Pharmaceut. Ass.
-Am. Conf. Pharmaceut.
-Chem. Soc.
+Am. Conf. Pharmaceut. Faculties
+Chem. Soc
 Ohio Pharmaceut. Ass.</t>
         </is>
       </c>
-      <c r="Q44" s="13" t="inlineStr">
+      <c r="Q44" s="5" t="inlineStr">
         <is>
           <t>Pharmacy food and drug laws; poison and habit-forming drug legislation</t>
         </is>
       </c>
-      <c r="R44" s="13" t="n"/>
-      <c r="S44" s="13" t="inlineStr"/>
+      <c r="R44" s="5" t="n"/>
+      <c r="S44" s="5" t="inlineStr">
+        <is>
+          <t>WARN: no_current_position -- no italic 1927 role: panel years to 1927 will be blank</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="6" t="n">
@@ -4392,7 +4396,7 @@
       </c>
       <c r="O45" s="9" t="inlineStr">
         <is>
-          <t>Collaborator, Plant Disease Surv, undated  [current 1927]</t>
+          <t>Collaborator, Plant Disease Surv, undated</t>
         </is>
       </c>
       <c r="P45" s="9" t="inlineStr">
@@ -4459,8 +4463,7 @@
       </c>
       <c r="M46" s="5" t="inlineStr">
         <is>
-          <t>A.B, ?, undated
-M.E, Va. Polytech, 1886</t>
+          <t>A.B, M.E. Va. Polytech, 1886</t>
         </is>
       </c>
       <c r="N46" s="5" t="inlineStr">
@@ -4484,7 +4487,7 @@
       <c r="R46" s="5" t="n"/>
       <c r="S46" s="5" t="inlineStr">
         <is>
-          <t>WARN: degree_missing_institution_and_year -- degree 'A.B' has neither institution nor year -- it may share its neighbour's printed ones
+          <t>WARN: degree_glued_into_institution -- institution 'M.E. Va. Polytech' starts with a degree abbreviation -- two printed degrees were probably fused into one
 WARN: no_current_position -- no italic 1927 role: panel years to 1927 will be blank</t>
         </is>
       </c>
@@ -4548,7 +4551,7 @@
       </c>
       <c r="N47" s="9" t="inlineStr">
         <is>
-          <t>Fellow, Earlham, 1896-1897
+          <t>Fellow, Haverford, 1896-1897
 Fellow, Chicago, 1901-1902
 Instr. math, Mich. State Col, 1897-1900
 Instr. math, Chicago Manual Training High Sch, 1902-1903
@@ -4562,8 +4565,8 @@
       <c r="P47" s="9" t="inlineStr">
         <is>
           <t>A.A.
-Astron. Soc.
-Math. Soc.
+Astron. Soc
+Math. Soc
 Soc. astron. de France</t>
         </is>
       </c>
@@ -4640,13 +4643,12 @@
       </c>
       <c r="O48" s="13" t="inlineStr">
         <is>
-          <t>Biol. surv, Colo, 1914
-In charge annual entom. collecting parties, Kansas, undated  [current 1927]</t>
+          <t>In charge annual entom. collecting parties, Biol. surv, Colo, 1914</t>
         </is>
       </c>
       <c r="P48" s="13" t="inlineStr">
         <is>
-          <t>Entom. Soc.</t>
+          <t>Kans. Entom. Soc.</t>
         </is>
       </c>
       <c r="Q48" s="13" t="inlineStr">
@@ -4726,13 +4728,13 @@
       </c>
       <c r="Q49" s="5" t="inlineStr">
         <is>
-          <t>The measurement of very short time intervals; time interval between the first appearance of spectrum lines; between excitation and fluorescent emission</t>
+          <t>The measurement of very short time intervals; time interval between the first appearance of spectrum lines, between excitation and fluorescent emission</t>
         </is>
       </c>
       <c r="R49" s="5" t="n"/>
       <c r="S49" s="5" t="inlineStr">
         <is>
-          <t>WARN: birth_field_repaired -- birth_date 'January 25, 1898' stripped (no printed trace); birth_year stripped too
+          <t>WARN: birth_field_repaired -- birth_date 'April 1, 1898' stripped (no printed trace); birth_year stripped too
 WARN: no_birth_year</t>
         </is>
       </c>
@@ -4800,7 +4802,8 @@
       <c r="O50" s="13" t="inlineStr"/>
       <c r="P50" s="13" t="inlineStr">
         <is>
-          <t>Wash. Biol. Soc.</t>
+          <t>Wash. Biol. Soc
+Fisheries Soc</t>
         </is>
       </c>
       <c r="Q50" s="13" t="inlineStr">
@@ -4867,7 +4870,6 @@
       <c r="M51" s="9" t="inlineStr">
         <is>
           <t>A.B, Nebraska, 1899
-study, Chicago, undated
 Ph.D, Columbia, 1912</t>
         </is>
       </c>
@@ -4950,9 +4952,9 @@
       <c r="N52" s="5" t="inlineStr">
         <is>
           <t>Asst. geol, Wisconsin, 1908-1909
-Instr, Wisconsin, 1911-1915
-Asst. prof, Wisconsin, 1915-1917
-Geologist, Wis. Geol. Surv, 1911-  [current 1927]
+Instr. geol, Wisconsin, 1911-1915
+Asst. prof. geol, Wisconsin, 1915-1917
+Geologist, Wis. Geol. Surv, 1911
 Chief of parties, Wis. Geol. Surv, 1913-1915
 Asst. state geologist, Wisconsin, 1916-1925
 Acting state geologist, Wisconsin, 1925-1926
@@ -4961,7 +4963,7 @@
       </c>
       <c r="O52" s="5" t="inlineStr">
         <is>
-          <t>Asst, Nat. Geog. Soc. exped., Alaska, 1909-1910</t>
+          <t>Asst., Nat. Geog. Soc. exped. Alaska, 1909-1910</t>
         </is>
       </c>
       <c r="P52" s="5" t="inlineStr">
@@ -5048,12 +5050,12 @@
       <c r="N53" s="9" t="inlineStr">
         <is>
           <t>Asst. anat, Hopkins, 1904-1905
-Instr, Michigan, 1905-1907
-Asst. prof, Philippines, 1907-1908
-Assoc. prof, Philippines, 1908-1910
-Assoc. prof, Tulane, 1910-1914
-Prof, Tulane, 1914-1916
-Prof, Virginia, 1916-  [current 1927]</t>
+Instr. anat, Michigan, 1905-1907
+Asst. prof. anat, Philippines, 1907-1908
+Assoc. prof. anat, Philippines, 1908-1910
+Assoc. prof. anat, Tulane, 1910-1914
+Prof. anat, Tulane, 1914-1916
+Prof. anat, Virginia, 1916-  [current 1927]</t>
         </is>
       </c>
       <c r="O53" s="9" t="inlineStr">
@@ -5061,9 +5063,9 @@
           <t>Lecturer, Teachers' Assembly, Baguio, 1908
 Govt. investigator, Benguet Igorots, 1908
 Exec. committee, sect. H, A.A., 1925
-Chairman, sect. H, A.A., 1926
-Councilor, Anthrop. Ass., 1919
-Pres, New Orleans Acad., 1915</t>
+Chairman, Ass. Anat; Anthrop. Ass., 1926
+Councilor, Ass. Anat; Anthrop. Ass., 1919
+President, New Orleans Acad., 1915</t>
         </is>
       </c>
       <c r="P53" s="9" t="inlineStr">
@@ -5147,8 +5149,8 @@
         <is>
           <t>Instr. chem, Idaho, 1900-1903
 Instr. chem, Columbia, 1903-1911
-Asst. prof. and assoc. prof, Columbia, 1911-1921
-Prof, Columbia, 1921-  [current 1927]</t>
+Asst. prof. and assoc. prof. chem, Columbia, 1911-1921
+Prof. chem, Columbia, 1921-  [current 1927]</t>
         </is>
       </c>
       <c r="O54" s="13" t="inlineStr"/>
@@ -5228,7 +5230,7 @@
       <c r="N55" s="9" t="inlineStr">
         <is>
           <t>Instr. agr. chem. and soils, Ohio State, 1908-1910
-Asst. prof, Ohio State, 1910-1913
+Asst. prof. agr. chem. and soils, Ohio State, 1910-1913
 Prof. soils in charge soil investigations, West Virginia, 1914-1916
 Prof. agr. chem. and soils, Ohio State, 1916-  [current 1927]</t>
         </is>
@@ -5312,14 +5314,14 @@
       </c>
       <c r="O56" s="13" t="inlineStr">
         <is>
-          <t>In charge weights and measures exhibit, Panama-Pacific Expos, 1915
+          <t>In charge weights and measures exhibit, Panama-Pacific Expos., 1915
 Sec'y, Nat. Screw Thread Commission, undated  [current 1927]</t>
         </is>
       </c>
       <c r="P56" s="13" t="inlineStr">
         <is>
           <t>Wash. Acad
-Wash. Philos. Soc.</t>
+Wash. Philos. Soc</t>
         </is>
       </c>
       <c r="Q56" s="13" t="inlineStr">
@@ -5389,16 +5391,19 @@
         <is>
           <t>Instr. chem, Wisconsin, 1919-1920
 Asst. technologist, Bur. Fisheries, 1920-1924
-Chief technologist, Bur. Fisheries, 1924-  [current 1927]
-Chemist, Colo. State Oil Lab, 1916
-Asst, Colorado, 1916-1917
+Chief technologist, Bur. Fisheries, 1924-  [current 1927]</t>
+        </is>
+      </c>
+      <c r="O57" s="9" t="inlineStr">
+        <is>
+          <t>Chemist, Colo. State Oil Lab, 1916
+Asst., Colorado, 1916-1917
 Chemist, Wilson and Co, 1920
 Asst. chemist, Puget Sound Navy Yard, 1917
 Ordnance dept, U.S.A., 1917-1919
-Research chemist, U.S.A., 1919</t>
-        </is>
-      </c>
-      <c r="O57" s="9" t="inlineStr"/>
+Research chemist, 1919</t>
+        </is>
+      </c>
       <c r="P57" s="9" t="inlineStr">
         <is>
           <t>Chem. Soc.</t>
@@ -5550,18 +5555,18 @@
       </c>
       <c r="M59" s="9" t="inlineStr">
         <is>
-          <t>C.E, E.M, Columbia, 1877</t>
+          <t>C.E, Columbia, 1877
+E.M, Columbia, 1877</t>
         </is>
       </c>
       <c r="N59" s="9" t="inlineStr">
         <is>
           <t>Asst. engineer, N. Y. and Brooklyn Bridge, 1877-1880
 Asst. and div. eng, C. B. and Q. Ry, 1880-1883
-Asst, U. S. Dept. Min. Surv, 1883-1885
+Asst., U. S. Dept. Min. Surv, 1883-1885
 Mining engineer, Ottumwa Fuel Co. and Colo. Fuel and Iron Co, 1885-1896
-Prin. sch. mines, Int. Correspondence Schools, undated
-Assoc. ed., Mines and Minerals, Int. Correspondence Schools, 1896-1911
-Senior assoc. ed., Coal Age, Int. Correspondence Schools, 1911-  [current 1927]</t>
+Prin. sch. mines, Int. Correspondence Schools, 1896-1911
+Senior assoc. ed., 'Coal Age', Int. Correspondence Schools, 1911-  [current 1927]</t>
         </is>
       </c>
       <c r="O59" s="9" t="inlineStr"/>
@@ -5642,18 +5647,18 @@
       <c r="N60" s="13" t="inlineStr">
         <is>
           <t>Instr. pharmacy, North Carolina, 1909-1913
-Asst. prof, North Carolina, 1913-1917
-Assoc. prof, North Carolina, 1917-1919
-Prof, North Carolina, 1919-  [current 1927]
+Asst. prof. pharmacy, North Carolina, 1913-1917
+Assoc. prof. pharmacy, North Carolina, 1917-1919
+Prof. pharmacy, North Carolina, 1919-  [current 1927]
 Sec'y, sch. pharmacy, North Carolina, 1916-  [current 1927]</t>
         </is>
       </c>
       <c r="O60" s="13" t="inlineStr">
         <is>
-          <t>Local sec'y, Pharmaceut. Ass., 1923
-Chairman, sect. educ. and legislation, Pharmaceut. Ass., 1925
-V. pres, Ass. Col. Pharm., 1925
-Pres, Elisha Mitchell Sci. Soc., 1917-1919
+          <t>Local sec'y, 1923
+Chairman, sect. educ. and legislation, 1925
+Vice president, Ass. Col. Pharm., 1925
+President, Elisha Mitchell Sci. Soc., 1919
 Sec'y-treas, N. C. Pharm. Ass., 1912-  [current 1927]</t>
         </is>
       </c>
@@ -5895,28 +5900,23 @@
       <c r="N63" s="9" t="inlineStr">
         <is>
           <t>Prof. physiol, Minnesota, 1888-1913
-Head dept, Minnesota, 1888-1909
-Head dept. physiol. and pharmacol, Minnesota, 1909-1913
+Head dept. physiol. and pharmacol, Minnesota, 1888-1909
 Assoc. prof. physiol, Minnesota, 1913-1925
-Emer. prof, Minnesota, 1925-  [current 1927]</t>
+Emer. prof., Minnesota, 1925-  [current 1927]
+Sec'y, med. sch, Minnesota, 1888-1925</t>
         </is>
       </c>
       <c r="O63" s="9" t="inlineStr">
         <is>
-          <t>Sec'y, med. sch, Minnesota, 1888-1925
-Member, Minn. Pure Water Commission, undated
-Sec'y, Minn. Acad. Med., 1890-1903
-Pres, Minn. Acad. Med., 1905
+          <t>Hon. Minn. Pure Water Commission, undated
+Hon. Am. Med. Ass., undated
+Hon. fel., Minn. Acad. Med., undated
+Sec'y, Minn. Acad. Med., 1900-1903
+President, Minn. Acad. Med., 1905
 Exec. sec'y, Hennepin County Pub. Health Ass., undated  [current 1927]</t>
         </is>
       </c>
-      <c r="P63" s="9" t="inlineStr">
-        <is>
-          <t>Am. Med. Ass.
-Minn. Acad. Med.
-Hennepin County Pub. Health Ass.</t>
-        </is>
-      </c>
+      <c r="P63" s="9" t="inlineStr"/>
       <c r="Q63" s="9" t="inlineStr">
         <is>
           <t>Nutrition; foods; food adulteration</t>
@@ -5986,14 +5986,18 @@
 Senior master, Asheville Sch, 1901-1920</t>
         </is>
       </c>
-      <c r="O64" s="5" t="inlineStr"/>
+      <c r="O64" s="5" t="inlineStr">
+        <is>
+          <t>Trustee, Ohio Acad., 1897-1900
+Sec'y, Ohio Acad., undated  [current 1927]</t>
+        </is>
+      </c>
       <c r="P64" s="5" t="inlineStr">
         <is>
           <t>A.A.
 Bot. Soc.
 Torrey Bot. Club
 Phytopath. Soc.
-Ohio Acad. (trustee, 97-00)
 N. C. Acad.</t>
         </is>
       </c>
@@ -6066,14 +6070,14 @@
       <c r="N65" s="9" t="inlineStr">
         <is>
           <t>Asst. engineer, sanit. dist, Chicago, 1892-1898
-Asst. engineer, Deep Waterway Commission, 1898-1900
-Canal and harbor works, C.Eng, U.S.A, 1900-1902
-Consulting engineer, Philippine Commission, 1902-1908
+Engineer, Deep Waterway Commission, 1898-1900
+Canal and harbor works, C.Eng., U.S.A., 1900-1902
+Consulting engineer, Philippine Commission, undated
 Director pub. works, P. I, 1902-1908
 Investigator of irrig, Java, Burma, India and Egypt, 1908-1909
 Chief engineer, P. R. Irrig. Service, 1910-1916
-Consulting engineer, ordnance dept, U.S.A, 1918
-Asst. chief eng. surveys, Grand Canal, China, 1918
+Consulting engineer, ordnance dept, U.S.A., 1918
+Asst. chief eng. surveys, Grand Canal, China, 1918-1919
 Engineer mem. highway commission, Panama, 1920-1921
 Consulting engineer, 1921-1924
 Designing engineer, Syracuse Int. Sewer Board, 1925-1926
@@ -6083,8 +6087,7 @@
       <c r="O65" s="9" t="inlineStr"/>
       <c r="P65" s="9" t="inlineStr">
         <is>
-          <t>Civil Eng
-West. Soc. Eng.</t>
+          <t>West. Soc. Eng.</t>
         </is>
       </c>
       <c r="Q65" s="9" t="n"/>
@@ -6152,11 +6155,10 @@
       </c>
       <c r="N66" s="13" t="inlineStr">
         <is>
-          <t>Instr. high sch, Wis, 1908-1910
+          <t>Instr. high sch, Wisconsin, 1908-1910
 Asst. chemist, forest products lab, U. S. Forest Service, Madison, 1910-1911
 Instr. chem, Kansas, 1912-1914
-Research chemist, Wyoming, 1914-  [current 1927]
-Plant investigator, Midwest Ref. Co, 1920</t>
+Research chemist, Wyoming, 1914-  [current 1927]</t>
         </is>
       </c>
       <c r="O66" s="13" t="inlineStr">
@@ -6246,13 +6248,14 @@
           <t>Research chemist, Am. Writing Paper Co, 1916
 Asst. chem, Mass. Inst. Tech, 1917-1918
 Research assoc, Mass. Inst. Tech, 1920-1923
-Asst. prof. physical chem., research, Mass. Inst. Tech, 1923-  [current 1927]</t>
+Research, Mass. Inst. Tech, 1923-  [current 1927]
+Asst. prof. physical chem. research, Mass. Inst. Tech, 1923-  [current 1927]</t>
         </is>
       </c>
       <c r="O67" s="9" t="inlineStr">
         <is>
           <t>Fellow, Mass. Inst. Tech, 1919-1920
-Nat. Research Council fellow chem, 1921-1923
+Fellow chem, Nat. Research Council, 1921-1923
 Cryogenic lab, Leiden, Holland, 1922-1923</t>
         </is>
       </c>
@@ -6332,11 +6335,12 @@
       <c r="N68" s="13" t="inlineStr">
         <is>
           <t>Instr. high sch, Colo, 1896-1897
-Wyo. bot, Wash. Col, 1899-1903
-Prof. and head dept. and botanist, Exp. Sta, Wash. Col, 1903-1912
+Instr. high sch, Wyo, 1898-1899
+Instr. bot, Wash. Col, 1899-1903
+Prof. and head dept. and botanist, Exp. Sta, 1903-1912
 Forest pathologist, U. S. Dept. Agr, 1912-1914
-Path. inspector, fed. hort. board, U. S. Dept. Agr, 1914-1919
-Pathologist in charge for. plant quarantines, U. S. Dept. Agr, 1919-  [current 1927]</t>
+Path. inspector, Fed. hort. board, 1914-1919
+Pathologist in charge for. plant quarantines, Fed. hort. board, 1919-  [current 1927]</t>
         </is>
       </c>
       <c r="O68" s="13" t="inlineStr">
@@ -6350,7 +6354,7 @@
           <t>A.A.
 Bot. Soc.
 Phytopath. Soc.
-Wash. Bot. Soc. (pres, 25)
+Wash. Bot. Soc.
 Wash. Acad.</t>
         </is>
       </c>
@@ -6413,7 +6417,8 @@
       </c>
       <c r="M69" s="9" t="inlineStr">
         <is>
-          <t>B.S, M.S, Ohio State, undated</t>
+          <t>B.S, Ohio State, 1896
+M.S, Ohio State, 1898</t>
         </is>
       </c>
       <c r="N69" s="9" t="inlineStr">
@@ -6429,7 +6434,7 @@
         <is>
           <t>Soc. Hort. Sci.
 Am. Peat Soc.
-Vegetable Growers Ass. (v. pres)
+Vegetable Growers Ass.
 Wash. Biol. Soc.
 Wash. Biol. Field Club</t>
         </is>
@@ -6589,11 +6594,14 @@
         <is>
           <t>Asst. anal. chem, Columbia, 1918-1921
 Research chemist, Firestone Tire and Rubber Co, 1922-1923
-Assoc. director research, Combustion Utilities Corp, 1923-  [current 1927]
-Research chemist, Gas W. S, 1917-1919</t>
-        </is>
-      </c>
-      <c r="O71" s="9" t="inlineStr"/>
+Assoc. director research, Combustion Utilities Corp, 1923-  [current 1927]</t>
+        </is>
+      </c>
+      <c r="O71" s="9" t="inlineStr">
+        <is>
+          <t>Research chemist, Gas W. S., 1917-1919</t>
+        </is>
+      </c>
       <c r="P71" s="9" t="inlineStr"/>
       <c r="Q71" s="9" t="inlineStr">
         <is>
@@ -6738,6 +6746,7 @@
       <c r="M73" s="9" t="inlineStr">
         <is>
           <t>B.S, Nebraska, 1920
+study, Nebraska, 1921-1923
 Ph.D, Nebraska, 1925
 study, Harvard Med. Sch, 1925</t>
         </is>
@@ -6747,11 +6756,7 @@
           <t>Instr. biochem, Nebraska, 1925-  [current 1927]</t>
         </is>
       </c>
-      <c r="O73" s="9" t="inlineStr">
-        <is>
-          <t>Fellow, Nebraska, 1921-1923</t>
-        </is>
-      </c>
+      <c r="O73" s="9" t="inlineStr"/>
       <c r="P73" s="9" t="inlineStr">
         <is>
           <t>A.A.
@@ -6827,14 +6832,14 @@
       </c>
       <c r="N74" s="13" t="inlineStr">
         <is>
-          <t>Dept. animal indust, U. S. Dept. Agr, 1911-1913
-Dept. dairy husbandry, Pa. State, 1913-1926
+          <t>Dept. dairy husbandry, Pa. State, 1913-1926
 Prof. dairy production in charge research, Pa. State, 1926-  [current 1927]</t>
         </is>
       </c>
       <c r="O74" s="13" t="inlineStr">
         <is>
-          <t>Shevlin fellow, Minnesota, 1922-1923</t>
+          <t>Shevlin fellow, Minnesota, 1922-1923
+Bur. animal indust, U. S. Dept. Agr, 1911-1913</t>
         </is>
       </c>
       <c r="P74" s="13" t="inlineStr">
@@ -6907,7 +6912,8 @@
       <c r="M75" s="5" t="inlineStr">
         <is>
           <t>B.S, Chicago, 1906
-Ph.D, Northwestern, 1909
+study, Chicago, 1906
+Ph.D, Chicago, 1909
 M.D, Northwestern, 1915</t>
         </is>
       </c>
@@ -7003,11 +7009,11 @@
       </c>
       <c r="N76" s="13" t="inlineStr">
         <is>
-          <t>Teacher and prin. schools, Pa., 1903-1908
+          <t>Teacher and prin., schools, Pa., 1903-1908
 Asst. instr. bot., Pa. State, 1913
 Instr. bot., Pa. State, 1914
-Instr. bot., N. Y. State Col. Agr., Cornell, 1914-1920
-Prof. bot., Wabash, 1920-  [current 1927]</t>
+Instr., N. Y. State Col. Agr., Cornell, 1914-1920
+Prof., Wabash, 1920-  [current 1927]</t>
         </is>
       </c>
       <c r="O76" s="13" t="inlineStr"/>
@@ -7072,7 +7078,7 @@
       </c>
       <c r="K77" s="8" t="inlineStr">
         <is>
-          <t>November 8, 1894</t>
+          <t>Nov. 8, 1894</t>
         </is>
       </c>
       <c r="L77" s="6" t="n">
@@ -7088,13 +7094,16 @@
         <is>
           <t>Res. house officer, Hopkins Hosp., 1921-1922
 Res. surgeon, New Haven Hosp., 1922-1923
-Arthur Tracy Cabot fellow, Harvard Med. Sch., 1923-1924
 Assoc. surg., Peter Bent Brigham Hosp., 1923-1924
 G. W. Crile fellow, sch. med., Western Reserve, 1924-1925
 Instr. surg. and res. surgeon, Lakeside Hosp., 1925-  [current 1927]</t>
         </is>
       </c>
-      <c r="O77" s="9" t="inlineStr"/>
+      <c r="O77" s="9" t="inlineStr">
+        <is>
+          <t>Arthur Tracy Cabot fellow, Harvard Med. Sch., undated</t>
+        </is>
+      </c>
       <c r="P77" s="9" t="inlineStr"/>
       <c r="Q77" s="9" t="inlineStr">
         <is>
@@ -7151,7 +7160,7 @@
       </c>
       <c r="K78" s="12" t="inlineStr">
         <is>
-          <t>September 26, 1870</t>
+          <t>Sept. 26, 1870</t>
         </is>
       </c>
       <c r="L78" s="10" t="n">
@@ -7165,24 +7174,22 @@
       <c r="N78" s="13" t="inlineStr">
         <is>
           <t>Assoc. prof. oto-laryngol., col. med., Illinois, 1904-  [current 1927]
-Attending surgeon, Cook Co. Hosp., 1905-  [current 1927]
+Attending surgeon, Cook Co. Hosp., 1905
 Head dept. ear, nose and throat, North Chicago Hosp., 1904-  [current 1927]</t>
         </is>
       </c>
       <c r="O78" s="13" t="inlineStr">
         <is>
-          <t>Lieut-col., Czecho-Slovak Army, 1918-1919</t>
-        </is>
-      </c>
-      <c r="P78" s="13" t="inlineStr">
-        <is>
-          <t>Am. Med. Ass. (pres. sect. oto-laryngol., 19)
-Otol. Soc.
-Acad. Ophthal. and Oto-Laryngol. (pres., 14)
-Laryngol., Rhinol. and Otol. Soc.
-Chicago Oto-Laryngol. Soc. (pres., 09)</t>
-        </is>
-      </c>
+          <t>Czecho-Slovak Army, 1918-1919
+Lieut-col., M.R.C., 1919
+Col. Surg., Am. Med. Ass. (pres., sect. oto-laryngol., 19), undated
+Pres., Otol. Soc., undated
+Pres., Acad. Ophthal. and Oto-Laryngol., 1914
+Pres., Laryngol., Rhinol. and Otol. Soc., undated
+Pres., Chicago Oto-Laryngol. Soc., 1909</t>
+        </is>
+      </c>
+      <c r="P78" s="13" t="inlineStr"/>
       <c r="Q78" s="13" t="inlineStr">
         <is>
           <t>Surgery of the head and neck</t>
@@ -7250,7 +7257,7 @@
       <c r="N79" s="9" t="inlineStr">
         <is>
           <t>Instr. mech. eng., North Dakota, 1904-1906
-Asst. prof. mech. eng., North Dakota, 1906-1907
+Asst. prof., North Dakota, 1906-1907
 Prof. applied math., North Dakota, 1907-1919
 Sec'y-treas., Ohio Valley Roofing Co., 1920-  [current 1927]</t>
         </is>
@@ -7317,7 +7324,7 @@
       </c>
       <c r="K80" s="12" t="inlineStr">
         <is>
-          <t>December 5, 1896</t>
+          <t>Dec. 5, 1896</t>
         </is>
       </c>
       <c r="L80" s="10" t="n">
@@ -7388,7 +7395,7 @@
       </c>
       <c r="K81" s="8" t="inlineStr">
         <is>
-          <t>February 2, 1889</t>
+          <t>Feb. 2, 1889</t>
         </is>
       </c>
       <c r="L81" s="6" t="n">
@@ -7471,7 +7478,7 @@
       </c>
       <c r="K82" s="12" t="inlineStr">
         <is>
-          <t>January 24, 1897</t>
+          <t>Jan. 24, 1897</t>
         </is>
       </c>
       <c r="L82" s="10" t="n">
@@ -7551,7 +7558,7 @@
       </c>
       <c r="K83" s="8" t="inlineStr">
         <is>
-          <t>January 11, 1875</t>
+          <t>Jan. 11, 1875</t>
         </is>
       </c>
       <c r="L83" s="6" t="n">
@@ -7566,12 +7573,12 @@
       </c>
       <c r="N83" s="9" t="inlineStr">
         <is>
-          <t>Engineer, Westinghouse Elec. and Mfg. Co., 1895-1896
-Engineer, Acker Process Co., 1896-1898
-Engineer, Acker Process Co., 1899-1900
-Engineer, Ampere Electrochem. Co., 1902-1903
-Engineer, Niagara Research Laboratories, 1903-1906
-Engineer, Electro Metal. Co. and Union Carbide Co., 1906-  [current 1927]</t>
+          <t>Westinghouse Elec. and Mfg. Co., Westinghouse Elec. and Mfg. Co., 1895-1896
+Acker Process Co., Acker Process Co., 1896-1898
+Acker Process Co., Acker Process Co., 1899-1900
+Ampere Electrochem. Co., Ampere Electrochem. Co., 1902-1903
+Niagara Research Laboratories, Niagara Research Laboratories, 1903-1906
+Electro Metal. Co. and Union Carbide Co., Electro Metal. Co. and Union Carbide Co., 1906-  [current 1927]</t>
         </is>
       </c>
       <c r="O83" s="9" t="inlineStr"/>
@@ -7579,7 +7586,7 @@
         <is>
           <t>Min. and Metal. Eng.
 Soc. Test. Mat.
-Electrochem. Soc. (pres., 25)
+Electrochem. Soc.
 Ceramic Soc.
 Chem. Soc.
 Min. and Metal. Soc.
@@ -7653,18 +7660,19 @@
       <c r="N84" s="13" t="inlineStr">
         <is>
           <t>Assoc. prof. math., Purdue, 1905-1912
-Actuary, State Life Ins. Co., 1912-  [current 1927]</t>
+Actuary, State Life Ins. Co., 1912-  [current 1927]
+Consulting actuary, undated  [current 1927]</t>
         </is>
       </c>
       <c r="O84" s="13" t="inlineStr">
         <is>
-          <t>Consulting actuary, undated  [current 1927]</t>
+          <t>Pres., Am. Inst. Actuaries, 1917-1919</t>
         </is>
       </c>
       <c r="P84" s="13" t="inlineStr">
         <is>
           <t>Math. Soc.
-Am. Inst. Actuaries (pres., 17-19)
+Am. Inst. Actuaries
 Statist. Ass.
 Actuarial science</t>
         </is>
@@ -7720,7 +7728,7 @@
       </c>
       <c r="K85" s="8" t="inlineStr">
         <is>
-          <t>September 19, 1883</t>
+          <t>Sept. 19, 1883</t>
         </is>
       </c>
       <c r="L85" s="6" t="n">
@@ -7771,7 +7779,7 @@
       </c>
       <c r="F86" s="12" t="inlineStr">
         <is>
-          <t>Stanford</t>
+          <t>Stanford University</t>
         </is>
       </c>
       <c r="G86" s="12" t="inlineStr">
@@ -7796,7 +7804,7 @@
       </c>
       <c r="K86" s="12" t="inlineStr">
         <is>
-          <t>January 4, 1895</t>
+          <t>Jan. 4, 1895</t>
         </is>
       </c>
       <c r="L86" s="10" t="n">
@@ -7819,7 +7827,7 @@
       </c>
       <c r="O86" s="13" t="inlineStr">
         <is>
-          <t>Consultant, bur. chem., U. S. Dept. Agr., 1924-1925</t>
+          <t>Consultant, Bur. Chem., U. S. Dept. Agr., 1924-1925</t>
         </is>
       </c>
       <c r="P86" s="13" t="inlineStr">
@@ -7888,7 +7896,7 @@
       </c>
       <c r="K87" s="8" t="inlineStr">
         <is>
-          <t>August 14, 1892</t>
+          <t>Aug. 14, 1892</t>
         </is>
       </c>
       <c r="L87" s="6" t="n">
@@ -7911,7 +7919,7 @@
       <c r="P87" s="9" t="inlineStr"/>
       <c r="Q87" s="9" t="inlineStr">
         <is>
-          <t>Synergism; colonic anaesthesia; ferment action</t>
+          <t>Synergism; colonic anesthesia; ferment action</t>
         </is>
       </c>
       <c r="R87" s="9" t="n"/>
@@ -7960,7 +7968,7 @@
       </c>
       <c r="K88" s="12" t="inlineStr">
         <is>
-          <t>February 15, 1888</t>
+          <t>Feb. 15, 1888</t>
         </is>
       </c>
       <c r="L88" s="10" t="n">
@@ -7976,15 +7984,15 @@
         <is>
           <t>Instrument man, Chicago and Northwest. Ry., 1912-1913
 Eng. inspector, Railroad Commission, Wis., 1913-1916
-Hydraulic engineer, water resources branch, U. S. Geol. Surv., 1916-1919
-Engineer, Cent. States Eng. Co., Iowa, 1919-1923
+Hydraulic engineer, Water resources branch, U. S. Geol. Surv., 1916-1919
+Engineer, Cent. States Eng. Co., 1919-1923
 Dist. engineer, water resources branch, U. S. Geol. Surv., Mo. and Ark., 1923-  [current 1927]</t>
         </is>
       </c>
       <c r="O88" s="13" t="inlineStr"/>
       <c r="P88" s="13" t="inlineStr">
         <is>
-          <t>A.A.</t>
+          <t>Assoc. Civil Eng.</t>
         </is>
       </c>
       <c r="Q88" s="13" t="inlineStr">
@@ -8059,7 +8067,7 @@
         <is>
           <t>Instr. physics, Purdue, 1905-1908
 Research asst., Clark, 1908-1909
-Prof., Mt. Allison, 1909-1911
+Prof., Mt. Allison, 1911-1912
 Instr., Syracuse, 1912-1914
 Instr., Northwestern, 1914-1915
 Instr., Pittsburgh, 1916-1917
@@ -8069,11 +8077,15 @@
       </c>
       <c r="O89" s="5" t="inlineStr">
         <is>
-          <t>Fellow, Northwestern, 1905
-A.A.S Physical Soc., undated  [current 1927]</t>
-        </is>
-      </c>
-      <c r="P89" s="5" t="inlineStr"/>
+          <t>Fellow, Northwestern, 1905</t>
+        </is>
+      </c>
+      <c r="P89" s="5" t="inlineStr">
+        <is>
+          <t>A.A.
+Physical Soc.</t>
+        </is>
+      </c>
       <c r="Q89" s="5" t="inlineStr">
         <is>
           <t>Residual E.M.F. in carbon arc; demagnetization of iron and steel; diffraction evolutes</t>
@@ -8135,20 +8147,17 @@
       <c r="L90" s="2" t="n"/>
       <c r="M90" s="5" t="inlineStr">
         <is>
-          <t>B.S. (E.E), Michigan, 1900
+          <t>B.S (E.E), Michigan, 1900
 M.M.E, Cornell, 1901</t>
         </is>
       </c>
       <c r="N90" s="5" t="inlineStr">
         <is>
-          <t>Prof. mech. eng., Utah, 1902-  [current 1927]</t>
-        </is>
-      </c>
-      <c r="O90" s="5" t="inlineStr">
-        <is>
-          <t>Engineer, Yampa tramway, Bingham, Utah, undated</t>
-        </is>
-      </c>
+          <t>Prof. mech. eng., Utah, 1902-  [current 1927]
+Engineer, Yampa tramway, Bingham, Utah, undated</t>
+        </is>
+      </c>
+      <c r="O90" s="5" t="inlineStr"/>
       <c r="P90" s="5" t="inlineStr">
         <is>
           <t>Mech. Eng.
@@ -8209,7 +8218,7 @@
       </c>
       <c r="J91" s="9" t="inlineStr">
         <is>
-          <t>Axtell, Nebr.</t>
+          <t>Axtell, Nebr</t>
         </is>
       </c>
       <c r="K91" s="8" t="inlineStr">
@@ -8231,7 +8240,8 @@
           <t>Instr. in charge petrol. tech, Oklahoma, 1922-1923
 Prof. and head petrol. eng, Colo. Sch. Mines, 1923-  [current 1927]
 Consulting engineer, 1922-  [current 1927]
-Lecturer, Denver Inst. Tech, 1925-  [current 1927]</t>
+Lecturer, Denver Inst. Tech, 1925
+Lecturer, Petrol. Inst, undated  [current 1927]</t>
         </is>
       </c>
       <c r="O91" s="9" t="inlineStr"/>
@@ -8286,7 +8296,7 @@
       </c>
       <c r="J92" s="13" t="inlineStr">
         <is>
-          <t>Grand Rapids, Mich.</t>
+          <t>Grand Rapids, Mich</t>
         </is>
       </c>
       <c r="K92" s="12" t="inlineStr">
@@ -8313,12 +8323,13 @@
       <c r="O92" s="13" t="inlineStr"/>
       <c r="P92" s="13" t="inlineStr">
         <is>
-          <t>A.A.</t>
+          <t>A.A.
+Phytopath. Soc.</t>
         </is>
       </c>
       <c r="Q92" s="13" t="inlineStr">
         <is>
-          <t>Phytopath. Soc. Grape root rot; cranberry diseases</t>
+          <t>Grape root rot; cranberry diseases</t>
         </is>
       </c>
       <c r="R92" s="13" t="n"/>
@@ -8362,7 +8373,7 @@
       </c>
       <c r="J93" s="9" t="inlineStr">
         <is>
-          <t>Olean, N. Y.</t>
+          <t>Olean, N. Y</t>
         </is>
       </c>
       <c r="K93" s="8" t="inlineStr">
@@ -8442,7 +8453,7 @@
       </c>
       <c r="J94" s="13" t="inlineStr">
         <is>
-          <t>Grand Rapids, Mich.</t>
+          <t>Grand Rapids, Mich</t>
         </is>
       </c>
       <c r="K94" s="12" t="inlineStr">
@@ -8526,7 +8537,7 @@
       </c>
       <c r="J95" s="9" t="inlineStr">
         <is>
-          <t>Hartford, Conn.</t>
+          <t>Hartford, Conn</t>
         </is>
       </c>
       <c r="K95" s="8" t="inlineStr">
@@ -8557,7 +8568,7 @@
       <c r="P95" s="9" t="inlineStr">
         <is>
           <t>A.A.
-Statistic Ass.
+Statist. Ass.
 Math. Soc.
 Math. Ass.</t>
         </is>
@@ -8608,7 +8619,7 @@
       </c>
       <c r="J96" s="13" t="inlineStr">
         <is>
-          <t>Utica, N. Y.</t>
+          <t>Utica, N. Y</t>
         </is>
       </c>
       <c r="K96" s="12" t="inlineStr">
@@ -8630,9 +8641,9 @@
       <c r="N96" s="13" t="inlineStr">
         <is>
           <t>Sci. asst, U. S. Dept. Agr, 1904-1907
-Asst. prof. bacter. and plant path, N. Dak. Col, 1907
+Asst. prof. bacter. and plant path, N. Dak. Col, undated
 Asst. botanist, Exp. Sta, 1907-1911
-Head dept. bacter, Oregon Col, 1911-1920
+Head dept. bacter, Oregon Col, undated
 Bacteriologist, Exp. Sta, 1911-1920
 Assoc. bacter, California, 1920-  [current 1927]</t>
         </is>
@@ -8704,7 +8715,7 @@
       </c>
       <c r="J97" s="9" t="inlineStr">
         <is>
-          <t>Brooklyn, N. Y.</t>
+          <t>Brooklyn, N. Y</t>
         </is>
       </c>
       <c r="K97" s="8" t="inlineStr">
@@ -8726,21 +8737,25 @@
         <is>
           <t>Instr. physics, Cornell, 1892-1893
 Asst. prof, Cornell, 1893-1904
-Prof, Cornell, 1904-  [current 1927]</t>
+Prof, Cornell, 1904-  [current 1927]
+Managing ed., 1913-1922</t>
         </is>
       </c>
       <c r="O97" s="9" t="inlineStr">
         <is>
           <t>Fellow, Cornell, 1891-1892
-Assoc. ed., 'Physical Rev', 1893-1912
-Managing ed., 'Physical Rev', 1913-1922</t>
+Assoc. ed., ‘Physical Rev’, 1893-1912
+Sec’y, A.A., B, 1897
+Sec’y, council, A.A., B, 1898
+Gen. sec’y, A.A., 1899
+Manager, Elec. Eng., 1914-1916
+V. pres., Elec. Eng., 1917</t>
         </is>
       </c>
       <c r="P97" s="9" t="inlineStr">
         <is>
-          <t>A.A. (sec'y, B, 97, sec'y, council, 98, gen. sec'y, 99)
-Physical Soc.
-Elec. Eng. (manager, 14-16, v. pres, 17)</t>
+          <t>A.A.
+Physical Soc.</t>
         </is>
       </c>
       <c r="Q97" s="9" t="inlineStr">
@@ -8793,7 +8808,7 @@
       </c>
       <c r="J98" s="13" t="inlineStr">
         <is>
-          <t>Racine, Wis.</t>
+          <t>Racine, Wis</t>
         </is>
       </c>
       <c r="K98" s="12" t="inlineStr">
@@ -8819,11 +8834,7 @@
 Director lab, Scovill Mfg. Co, 1925-  [current 1927]</t>
         </is>
       </c>
-      <c r="O98" s="13" t="inlineStr">
-        <is>
-          <t>Engineer, West. Elec. Co, 1919</t>
-        </is>
-      </c>
+      <c r="O98" s="13" t="inlineStr"/>
       <c r="P98" s="13" t="inlineStr">
         <is>
           <t>Elec. Eng.
@@ -8882,7 +8893,7 @@
       </c>
       <c r="J99" s="9" t="inlineStr">
         <is>
-          <t>Monson, Mass.</t>
+          <t>Monson, Mass</t>
         </is>
       </c>
       <c r="K99" s="8" t="inlineStr">
@@ -8961,7 +8972,7 @@
       </c>
       <c r="J100" s="5" t="inlineStr">
         <is>
-          <t>St. Johns, Mich.</t>
+          <t>St. Johns, Mich</t>
         </is>
       </c>
       <c r="K100" s="4" t="inlineStr">
@@ -9059,7 +9070,7 @@
       </c>
       <c r="J101" s="9" t="inlineStr">
         <is>
-          <t>Brooklyn, N. Y.</t>
+          <t>Brooklyn, N. Y</t>
         </is>
       </c>
       <c r="K101" s="8" t="inlineStr">
@@ -9083,7 +9094,7 @@
       </c>
       <c r="O101" s="9" t="inlineStr">
         <is>
-          <t>Cor. mem., London Zool. Soc, undated</t>
+          <t>Cor. mem., London Zool. Soc., undated</t>
         </is>
       </c>
       <c r="P101" s="9" t="inlineStr">
@@ -9091,11 +9102,11 @@
           <t>A.A.
 fel. Ornith. Union
 Soc. Mammal
-Ecol. Soc.
-N. Y. Linnean Soc.
-fel. N. Y. Zool. Soc.
-fel. N. Y. Acad.
-N. Y. Audubon Soc.</t>
+Ecol. Soc
+N. Y. Linnean Soc
+fel. N. Y. Zool. Soc
+fel. N. Y. Acad
+N. Y. Audubon Soc</t>
         </is>
       </c>
       <c r="Q101" s="9" t="inlineStr">
@@ -9144,7 +9155,7 @@
       </c>
       <c r="J102" s="13" t="inlineStr">
         <is>
-          <t>Mason City, Iowa.</t>
+          <t>Mason City, Iowa</t>
         </is>
       </c>
       <c r="K102" s="12" t="inlineStr">
@@ -9232,7 +9243,7 @@
       </c>
       <c r="J103" s="9" t="inlineStr">
         <is>
-          <t>Raymond, N. H.</t>
+          <t>Raymond, N. H</t>
         </is>
       </c>
       <c r="K103" s="8" t="inlineStr">
@@ -9246,7 +9257,7 @@
       <c r="M103" s="9" t="inlineStr">
         <is>
           <t>B.S, Washburn, 1896
-A.M, Kansas, 1897
+A.M, Washburn, 1897
 Ph.D, Kansas, 1899</t>
         </is>
       </c>
@@ -9259,16 +9270,14 @@
 Assoc. prof, Indiana, 1909-1917
 Geologist, bur. econ. geol, Texas, 1917-1922
 Geologist, Empire Gas and Fuel Co, 1922-1924
-Geologist, Dixie Oil Co, 1924-  [current 1927]</t>
+Geologist, Dixie Oil Co, 1924-  [current 1927]
+Asst., Kans. Geol. Surv, 1896-1898
+Asst., U. S. Geol. Surv, 1901-1903</t>
         </is>
       </c>
       <c r="O103" s="9" t="inlineStr">
         <is>
-          <t>Asst., Kans. Geol. Surv, 1896
-Asst., Kans. Geol. Surv, 1898
-Asst., Kans. Geol. Surv, 1903-1909
-Asst., U. S. Geol. Surv, 1901-1903
-Exec. committee, A.A., 1916</t>
+          <t>Exec. committee, A.A., 1916</t>
         </is>
       </c>
       <c r="P103" s="9" t="inlineStr">
@@ -9336,7 +9345,7 @@
       </c>
       <c r="K104" s="12" t="inlineStr">
         <is>
-          <t>December 7, 1894</t>
+          <t>Dec. 7, 1894</t>
         </is>
       </c>
       <c r="L104" s="10" t="n">
@@ -9428,7 +9437,7 @@
       </c>
       <c r="M105" s="9" t="inlineStr">
         <is>
-          <t>A.B, Columbia, 1896
+          <t>study, Columbia, 1896
 M.D, Columbia, 1899</t>
         </is>
       </c>
@@ -9525,14 +9534,11 @@
       </c>
       <c r="N106" s="13" t="inlineStr">
         <is>
-          <t>Instr. biol, Yale, 1925-  [current 1927]</t>
-        </is>
-      </c>
-      <c r="O106" s="13" t="inlineStr">
-        <is>
-          <t>Instr, Woods Hole, 1924-1925</t>
-        </is>
-      </c>
+          <t>Instr. biol, Yale, 1925-  [current 1927]
+Instr, Woods Hole, 1924-1925</t>
+        </is>
+      </c>
+      <c r="O106" s="13" t="inlineStr"/>
       <c r="P106" s="13" t="inlineStr">
         <is>
           <t>Soc. Zool.</t>
@@ -9563,7 +9569,7 @@
       </c>
       <c r="E107" s="9" t="inlineStr">
         <is>
-          <t>State College, Pa</t>
+          <t>(Mrs. Warren Mack), State College, Pa</t>
         </is>
       </c>
       <c r="F107" s="8" t="inlineStr">
@@ -9593,7 +9599,7 @@
       </c>
       <c r="K107" s="8" t="inlineStr">
         <is>
-          <t>December 19, 1891</t>
+          <t>Dec. 19, 1891</t>
         </is>
       </c>
       <c r="L107" s="6" t="n">
@@ -9608,7 +9614,7 @@
       <c r="N107" s="9" t="inlineStr">
         <is>
           <t>Teacher, high sch, Mo, 1913-1915
-Head dept, Mo, 1915-1919
+Head dept, high sch, Mo, 1915-1919
 Instr. chem, Pa. State, 1919-1920
 Asst. prof, Pa. State, 1920-  [current 1927]</t>
         </is>
@@ -9675,7 +9681,7 @@
       </c>
       <c r="K108" s="12" t="inlineStr">
         <is>
-          <t>August 31, 1867</t>
+          <t>Aug. 31, 1867</t>
         </is>
       </c>
       <c r="L108" s="10" t="n">
@@ -9690,20 +9696,21 @@
       </c>
       <c r="N108" s="13" t="inlineStr">
         <is>
-          <t>Instr. physics and chemist, Alabama Geol. Surv, 1888-1889
-Research chemist, La. Exp. Sta, undated
+          <t>Instr. physics, Alabama, 1888-1889
+Chemist, Ala. Geol. Surv, 1888-1889
+Research chemist, La. Exp. Sta, 1893-1896
 Prof. chem, La. Sch. of Sugar, 1893-1896
 Prof. nat. science, Bethel, 1896-1897
-Prof. chem, Ga. State Col. for Women, 1897-  [current 1927]
+Chem, Ga. State Col. for Women, 1897-  [current 1927]
 Dean col. arts and sciences, Ga. State Col. for Women, 1925-  [current 1927]
-Chairman faculty, Ga. State Col. for Women, 1910-  [current 1927]</t>
+Chairman faculty, Ga. State Col. for Women, 1910-  [current 1927]
+Acting pres, Ga. State Col. for Women, 1922-1923
+Acting pres, Ga. State Col. for Women, 1927</t>
         </is>
       </c>
       <c r="O108" s="13" t="inlineStr">
         <is>
-          <t>Acting pres, Ga. State Col. for Women, 1922-1923
-Acting pres, Ga. State Col. for Women, 1927
-Summer prof, Georgia, 1909</t>
+          <t>Summer prof, Georgia, 1909</t>
         </is>
       </c>
       <c r="P108" s="13" t="inlineStr">
@@ -9714,10 +9721,14 @@
       </c>
       <c r="Q108" s="13" t="inlineStr">
         <is>
-          <t>Action of alcohol on certain diazo compounds; sugar chemistry; nitric nitrogen gathered by the Leguminosae</t>
-        </is>
-      </c>
-      <c r="R108" s="13" t="n"/>
+          <t>Action of alcohol on certain diazo compounds</t>
+        </is>
+      </c>
+      <c r="R108" s="13" t="inlineStr">
+        <is>
+          <t>Sugar chemistry; nitric nitrogen gathered by the Leguminosae</t>
+        </is>
+      </c>
       <c r="S108" s="13" t="inlineStr"/>
     </row>
     <row r="109">
@@ -9860,7 +9871,7 @@
       </c>
       <c r="K110" s="12" t="inlineStr">
         <is>
-          <t>January 21, 1886</t>
+          <t>Jan. 21, 1886</t>
         </is>
       </c>
       <c r="L110" s="10" t="n">
@@ -9963,7 +9974,7 @@
         <is>
           <t>Supt. schools, Iowa, 1889-1895
 Prof. physics and chem, Parsons, 1895-1899
-Prof. physics and chem, Iowa State Teachers Col, 1899-  [current 1927]</t>
+Prof. physics, Iowa State Teachers Col, 1899-  [current 1927]</t>
         </is>
       </c>
       <c r="O111" s="9" t="inlineStr"/>
@@ -10037,7 +10048,7 @@
       </c>
       <c r="M112" s="13" t="inlineStr">
         <is>
-          <t>M.D, Rush, 1907</t>
+          <t>M.D, ?, 1907</t>
         </is>
       </c>
       <c r="N112" s="13" t="inlineStr">
@@ -10048,17 +10059,17 @@
 Teaching fellow, Harvard Med. Sch, 1911-1912
 Instr. comp. anat, Harvard Med. Sch, 1913-1918
 Asst. dean, demonstrator anat. and instr. histol, Harvard Med. Sch, 1918-1921
-Prof. anat, Boston University School of Medicine, undated  [current 1927]
+Prof. anat, sch. med, Boston, 1921-  [current 1927]
 Dean, Boston University School of Medicine, 1923-  [current 1927]</t>
         </is>
       </c>
       <c r="O112" s="13" t="inlineStr">
         <is>
-          <t>Research assoc, Carnegie Institution, 1915
+          <t>Research assoc, Carnegie Institution, 1915-  [current 1927]
 Med. advisory council, Life Exten. Inst, undated
 Chairman committee educ, Ass. Am. Med. Col, 1924-  [current 1927]
 Chairman committee pub. health and sanitation, Boston Chamber of Commerce, undated
-U.S.A, 1917-1919</t>
+U.S.A., 1917-1919</t>
         </is>
       </c>
       <c r="P112" s="13" t="inlineStr">
@@ -10122,7 +10133,7 @@
       </c>
       <c r="K113" s="8" t="inlineStr">
         <is>
-          <t>December 22, 1886</t>
+          <t>Dec. 22, 1886</t>
         </is>
       </c>
       <c r="L113" s="6" t="n">
@@ -10199,7 +10210,7 @@
       </c>
       <c r="K114" s="12" t="inlineStr">
         <is>
-          <t>September 24, 1895</t>
+          <t>Sept. 24, 1895</t>
         </is>
       </c>
       <c r="L114" s="10" t="n">
@@ -10241,7 +10252,7 @@
       </c>
       <c r="B115" s="7" t="inlineStr">
         <is>
-          <t>Behre, Charles H(enry), Jr</t>
+          <t>Behre, Charles H(enry), Jr.</t>
         </is>
       </c>
       <c r="C115" s="6" t="inlineStr"/>
@@ -10305,8 +10316,8 @@
       </c>
       <c r="O115" s="9" t="inlineStr">
         <is>
-          <t>Asst. geologist, U. S. Geol. Surv, 1921
-Cooperative geologist, Pa. Geol. Surv, 1922</t>
+          <t>Asst. geologist, U. S. Geol. Surv, 1921-  [current 1927]
+Cooperative geologist, Pa. Geol. Surv, 1922-  [current 1927]</t>
         </is>
       </c>
       <c r="P115" s="9" t="inlineStr">
@@ -10371,7 +10382,7 @@
       </c>
       <c r="K116" s="12" t="inlineStr">
         <is>
-          <t>September 28, 1886</t>
+          <t>Sept. 28, 1886</t>
         </is>
       </c>
       <c r="L116" s="10" t="n">
@@ -10470,7 +10481,6 @@
         <is>
           <t>Research asst. bacter, Northwestern, 1919-1920
 Instr. chem., med. col, Cornell, 1922-1924
-Instr. chem., med. col, Cornell, 1925-  [current 1927]
 Research chemist, lab, Union Central Life Ins. Co, 1924-  [current 1927]</t>
         </is>
       </c>
@@ -10723,15 +10733,12 @@
       <c r="N120" s="13" t="inlineStr">
         <is>
           <t>Clin. prof. surg, Albany Med. Col, Union, 1914-  [current 1927]
-Asst. surgeon, Albany Hosp, undated  [current 1927]</t>
+Asst. surgeon, Albany Hosp, undated  [current 1927]
+Asst. Path. and Bact, undated  [current 1927]</t>
         </is>
       </c>
       <c r="O120" s="13" t="inlineStr"/>
-      <c r="P120" s="13" t="inlineStr">
-        <is>
-          <t>Ass. Path. and Bact.</t>
-        </is>
-      </c>
+      <c r="P120" s="13" t="inlineStr"/>
       <c r="Q120" s="13" t="inlineStr">
         <is>
           <t>Surgery; pathology and surgery of the thyroid gland</t>
@@ -10799,7 +10806,7 @@
           <t>Asst. chem. sect, Iowa Exp. Sta, 1906-1908
 Tobacco experiments, Iowa Exp. Sta, 1908-1909
 In charge plant improvement, Sunnybrook Tobacco Co, 1909-1910
-Asst. in charge New Eng. tobacco investigations, Bur. plant indust, U. S. Dept. Agr, 1911-1919
+Asst. in charge New Eng. tobacco investigations, Bur. Plant Indust, U. S. Dept. Agr, 1911-1919
 Asst. manager, H. Zering Mfg. Co, 1919-1922
 In charge farm dept. and advertising, Lippincott Co, 1922-1923
 Research, Flo.-Ga. Tobacco Growers Ass. and research work, Am. Sumatra and Wedeles Tobacco Companies, 1923-  [current 1927]</t>
@@ -10883,7 +10890,7 @@
       </c>
       <c r="N122" s="5" t="inlineStr">
         <is>
-          <t>Chemist, du Pont Eng. Co, Tenn, 1918
+          <t>Chemist, Du Pont Eng. Co, Tenn, 1918
 Asst. chem, Princeton, 1919-1922
 Asst. prof, Florida, 1922-1923
 Prof. chem. eng, Florida, 1923-  [current 1927]</t>
@@ -10891,7 +10898,7 @@
       </c>
       <c r="O122" s="5" t="inlineStr">
         <is>
-          <t>Van der Poel fellow, Rutgers, 1918-1919
+          <t>Van der Poel fellow, 1918-1919
 Summers, chemist, Noil Color and Chem. Co, 1920-1922
 Assoc. ed, Jour. Chem. Educ., 1924-1925
 Capt, C.W.S., undated</t>
@@ -10972,7 +10979,8 @@
       </c>
       <c r="N123" s="9" t="inlineStr">
         <is>
-          <t>Prof. bacter, Rush Med. Col, Chicago, 1891-1898
+          <t>Vienna, undated
+Prof. bacter, Rush Med. Col, Chicago, 1891-1898
 Genito-urinary surg, Rush Med. Col, Chicago, 1898-  [current 1927]</t>
         </is>
       </c>
@@ -10983,7 +10991,7 @@
       </c>
       <c r="P123" s="9" t="inlineStr">
         <is>
-          <t>A.A.
+          <t>A.A
 Ass. Genito-Urinary Surg. (pres, 02)
 Urol. Ass. (pres, 08)</t>
         </is>
@@ -11083,7 +11091,11 @@
           <t>Bell, E(lexious) T(hompson)</t>
         </is>
       </c>
-      <c r="C125" s="6" t="inlineStr"/>
+      <c r="C125" s="6" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
       <c r="D125" s="8" t="inlineStr">
         <is>
           <t>Prof.</t>
@@ -11130,7 +11142,8 @@
       <c r="M125" s="9" t="inlineStr">
         <is>
           <t>B.S, Missouri, 1901
-M.D, Missouri, 1903</t>
+M.D, Missouri, 1903
+study, Bonn, 1905-1906</t>
         </is>
       </c>
       <c r="N125" s="9" t="inlineStr">
@@ -11138,13 +11151,17 @@
           <t>Asst. anat, Missouri, 1902-1903
 Instr, Missouri, 1903-1907
 Asst. prof, Missouri, 1907-1911
-Path, Minnesota, 1911-1916
+Asst. prof. path, Minnesota, 1911-1916
 Assoc. prof, Minnesota, 1916-1920
 Prof, Minnesota, 1920-  [current 1927]
 Director dept, Minnesota, 1921-  [current 1927]</t>
         </is>
       </c>
-      <c r="O125" s="9" t="inlineStr"/>
+      <c r="O125" s="9" t="inlineStr">
+        <is>
+          <t>Fellow, Missouri, 1901-1902</t>
+        </is>
+      </c>
       <c r="P125" s="9" t="inlineStr">
         <is>
           <t>A.A.
@@ -11371,7 +11388,7 @@
       </c>
       <c r="J128" s="13" t="inlineStr">
         <is>
-          <t>Halifax</t>
+          <t>Halifax, N. S</t>
         </is>
       </c>
       <c r="K128" s="12" t="inlineStr">
@@ -11404,7 +11421,7 @@
       </c>
       <c r="P128" s="13" t="inlineStr">
         <is>
-          <t>A.A.
+          <t>A.A
 Bot. Soc
 British Ecol. Soc.</t>
         </is>
@@ -11429,7 +11446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -11487,7 +11504,7 @@
       </c>
       <c r="E2" s="15" t="inlineStr">
         <is>
-          <t>birth_date 'November 3, 1893' stripped (no printed trace)</t>
+          <t>birth_date 'Jan 3, 1893' stripped (no printed trace)</t>
         </is>
       </c>
     </row>
@@ -11570,7 +11587,7 @@
       </c>
       <c r="B6" s="15" t="inlineStr">
         <is>
-          <t>birth_month_ocr_mismatch</t>
+          <t>no_current_position</t>
         </is>
       </c>
       <c r="C6" s="15" t="n">
@@ -11578,12 +11595,12 @@
       </c>
       <c r="D6" s="15" t="inlineStr">
         <is>
-          <t>Bausch, Edward</t>
+          <t>Bawden, H(enry) Heath</t>
         </is>
       </c>
       <c r="E6" s="15" t="inlineStr">
         <is>
-          <t>extracted 'Oct. 26, 1854' but the OCR text layer reads 'Sept.26,54' -- verify the month on the page image</t>
+          <t>no italic 1927 role: panel years to 1927 will be blank</t>
         </is>
       </c>
     </row>
@@ -11595,20 +11612,20 @@
       </c>
       <c r="B7" s="15" t="inlineStr">
         <is>
-          <t>no_current_position</t>
+          <t>birth_month_ocr_mismatch</t>
         </is>
       </c>
       <c r="C7" s="15" t="n">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D7" s="15" t="inlineStr">
         <is>
-          <t>Bawden, H(enry) Heath</t>
+          <t>Beadle, C(hauncey) D(elos)</t>
         </is>
       </c>
       <c r="E7" s="15" t="inlineStr">
         <is>
-          <t>no italic 1927 role: panel years to 1927 will be blank</t>
+          <t>extracted 'January 5, 1866' but the OCR text layer reads 'Aug.5,66' -- verify the month on the page image</t>
         </is>
       </c>
     </row>
@@ -11620,7 +11637,7 @@
       </c>
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>birth_month_ocr_mismatch</t>
+          <t>no_current_position</t>
         </is>
       </c>
       <c r="C8" s="15" t="n">
@@ -11633,7 +11650,7 @@
       </c>
       <c r="E8" s="15" t="inlineStr">
         <is>
-          <t>extracted 'January 5, 1866' but the OCR text layer reads 'Aug.5,66' -- verify the month on the page image</t>
+          <t>no italic 1927 role: panel years to 1927 will be blank</t>
         </is>
       </c>
     </row>
@@ -11645,7 +11662,7 @@
       </c>
       <c r="B9" s="15" t="inlineStr">
         <is>
-          <t>no_current_position</t>
+          <t>birth_field_repaired</t>
         </is>
       </c>
       <c r="C9" s="15" t="n">
@@ -11653,12 +11670,12 @@
       </c>
       <c r="D9" s="15" t="inlineStr">
         <is>
-          <t>Beadle, C(hauncey) D(elos)</t>
+          <t>Beal, Carl H(ugh)</t>
         </is>
       </c>
       <c r="E9" s="15" t="inlineStr">
         <is>
-          <t>no italic 1927 role: panel years to 1927 will be blank</t>
+          <t>all birth fields cleared: birth_place 'A.B. Stanford' was degree text</t>
         </is>
       </c>
     </row>
@@ -11670,7 +11687,7 @@
       </c>
       <c r="B10" s="15" t="inlineStr">
         <is>
-          <t>birth_field_repaired</t>
+          <t>no_birth_year</t>
         </is>
       </c>
       <c r="C10" s="15" t="n">
@@ -11681,11 +11698,7 @@
           <t>Beal, Carl H(ugh)</t>
         </is>
       </c>
-      <c r="E10" s="15" t="inlineStr">
-        <is>
-          <t>all birth fields cleared: birth_place 'A.B. Stanford' was degree text</t>
-        </is>
-      </c>
+      <c r="E10" s="15" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="15" t="inlineStr">
@@ -11695,7 +11708,7 @@
       </c>
       <c r="B11" s="15" t="inlineStr">
         <is>
-          <t>no_birth_year</t>
+          <t>no_current_position</t>
         </is>
       </c>
       <c r="C11" s="15" t="n">
@@ -11703,10 +11716,14 @@
       </c>
       <c r="D11" s="15" t="inlineStr">
         <is>
-          <t>Beal, Carl H(ugh)</t>
-        </is>
-      </c>
-      <c r="E11" s="15" t="inlineStr"/>
+          <t>Beal, J(ames) H(artley)</t>
+        </is>
+      </c>
+      <c r="E11" s="15" t="inlineStr">
+        <is>
+          <t>no italic 1927 role: panel years to 1927 will be blank</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="15" t="inlineStr">
@@ -11716,7 +11733,7 @@
       </c>
       <c r="B12" s="15" t="inlineStr">
         <is>
-          <t>degree_missing_institution_and_year</t>
+          <t>degree_glued_into_institution</t>
         </is>
       </c>
       <c r="C12" s="15" t="n">
@@ -11729,7 +11746,7 @@
       </c>
       <c r="E12" s="15" t="inlineStr">
         <is>
-          <t>degree 'A.B' has neither institution nor year -- it may share its neighbour's printed ones</t>
+          <t>institution 'M.E. Va. Polytech' starts with a degree abbreviation -- two printed degrees were probably fused into one</t>
         </is>
       </c>
     </row>
@@ -11779,7 +11796,7 @@
       </c>
       <c r="E14" s="15" t="inlineStr">
         <is>
-          <t>birth_date 'January 25, 1898' stripped (no printed trace); birth_year stripped too</t>
+          <t>birth_date 'April 1, 1898' stripped (no printed trace); birth_year stripped too</t>
         </is>
       </c>
     </row>
@@ -12008,16 +12025,20 @@
       </c>
       <c r="B24" s="15" t="inlineStr">
         <is>
-          <t>star_mismatch</t>
+          <t>duplicate_degree_type</t>
         </is>
       </c>
       <c r="C24" s="15" t="n">
         <v>84</v>
       </c>
-      <c r="D24" s="15" t="inlineStr"/>
+      <c r="D24" s="15" t="inlineStr">
+        <is>
+          <t>Beisler, Walter H(erman)</t>
+        </is>
+      </c>
       <c r="E24" s="15" t="inlineStr">
         <is>
-          <t>page prints 2 asterisk(s) but 1 profile(s) came back starred: Bell</t>
+          <t>'M.S' listed 2 times -- check whether one is a degreeless study spell</t>
         </is>
       </c>
     </row>
@@ -12029,7 +12050,7 @@
       </c>
       <c r="B25" s="15" t="inlineStr">
         <is>
-          <t>duplicate_degree_type</t>
+          <t>no_current_position</t>
         </is>
       </c>
       <c r="C25" s="15" t="n">
@@ -12037,42 +12058,17 @@
       </c>
       <c r="D25" s="15" t="inlineStr">
         <is>
-          <t>Beisler, Walter H(erman)</t>
+          <t>Belknap, W(illiam) E(thelbert)</t>
         </is>
       </c>
       <c r="E25" s="15" t="inlineStr">
         <is>
-          <t>'M.S' listed 2 times -- check whether one is a degreeless study spell</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="15" t="inlineStr">
-        <is>
-          <t>WARN</t>
-        </is>
-      </c>
-      <c r="B26" s="15" t="inlineStr">
-        <is>
-          <t>no_current_position</t>
-        </is>
-      </c>
-      <c r="C26" s="15" t="n">
-        <v>84</v>
-      </c>
-      <c r="D26" s="15" t="inlineStr">
-        <is>
-          <t>Belknap, W(illiam) E(thelbert)</t>
-        </is>
-      </c>
-      <c r="E26" s="15" t="inlineStr">
-        <is>
           <t>no italic 1927 role: panel years to 1927 will be blank</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E26"/>
+  <autoFilter ref="A1:E25"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>